<commit_message>
Update Nexlev and Viomi input sheets
</commit_message>
<xml_diff>
--- a/data/input/inventory_snapshot_nexlev.xlsx
+++ b/data/input/inventory_snapshot_nexlev.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\inventory\Week 18\Nexlev\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58FD3A33-8E7A-4EE0-AD3B-53B7771E375D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -1583,40 +1583,6 @@
     </dxf>
     <dxf>
       <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -1771,6 +1737,8 @@
     </dxf>
     <dxf>
       <font>
+        <condense val="0"/>
+        <extend val="0"/>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -1781,48 +1749,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -2025,6 +1951,80 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -13426,91 +13426,91 @@
   </sheetData>
   <autoFilter ref="A1:L538" xr:uid="{76CBFB1B-DC23-4380-8138-4D6BFF18CBC5}"/>
   <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="A448:A449">
+    <cfRule type="duplicateValues" dxfId="57" priority="1597"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A455:A462">
+    <cfRule type="duplicateValues" dxfId="56" priority="1587"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="duplicateValues" dxfId="57" priority="1340"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="1340"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D448">
-    <cfRule type="duplicateValues" dxfId="56" priority="103"/>
-    <cfRule type="duplicateValues" dxfId="55" priority="104"/>
-    <cfRule type="duplicateValues" dxfId="54" priority="105" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="53" priority="106" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="103"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="104"/>
     <cfRule type="duplicateValues" dxfId="52" priority="107" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="106" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="105" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D449">
-    <cfRule type="duplicateValues" dxfId="51" priority="98"/>
-    <cfRule type="duplicateValues" dxfId="50" priority="99"/>
-    <cfRule type="duplicateValues" dxfId="49" priority="100" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="48" priority="101" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="47" priority="102" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="98"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="99"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="100" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="101" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="102" stopIfTrue="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D450:D454">
+    <cfRule type="duplicateValues" dxfId="44" priority="1596" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="1595" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="1594"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="1590"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="1593"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="1592"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="1591"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="1589"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D455:D456">
-    <cfRule type="duplicateValues" dxfId="46" priority="52"/>
-    <cfRule type="duplicateValues" dxfId="45" priority="53"/>
-    <cfRule type="duplicateValues" dxfId="44" priority="54" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="43" priority="55" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="42" priority="56" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="53"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="54" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="55" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="56" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="52"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D459">
-    <cfRule type="duplicateValues" dxfId="41" priority="47"/>
-    <cfRule type="duplicateValues" dxfId="40" priority="48"/>
-    <cfRule type="duplicateValues" dxfId="39" priority="49" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="38" priority="50" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="37" priority="51" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="48"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="51" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="50" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="49" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="47"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D460">
-    <cfRule type="duplicateValues" dxfId="36" priority="42"/>
-    <cfRule type="duplicateValues" dxfId="35" priority="43"/>
-    <cfRule type="duplicateValues" dxfId="34" priority="44" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="33" priority="45" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="32" priority="46" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="46" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="45" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="44" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="43"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="42"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D462">
-    <cfRule type="duplicateValues" dxfId="31" priority="25"/>
-    <cfRule type="duplicateValues" dxfId="30" priority="26"/>
-    <cfRule type="duplicateValues" dxfId="29" priority="27"/>
-    <cfRule type="duplicateValues" dxfId="28" priority="28"/>
-    <cfRule type="duplicateValues" dxfId="27" priority="29"/>
-    <cfRule type="duplicateValues" dxfId="26" priority="30"/>
-    <cfRule type="duplicateValues" dxfId="25" priority="31" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="24" priority="32" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="32" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="31" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="29"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D463:D465">
+    <cfRule type="duplicateValues" dxfId="13" priority="1570"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="1571"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="1572"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="1574"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="1575"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="1576" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="1577" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="1573"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:H1">
-    <cfRule type="duplicateValues" dxfId="23" priority="1551"/>
-    <cfRule type="duplicateValues" dxfId="22" priority="1552" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="1551"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="1552" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1">
-    <cfRule type="duplicateValues" dxfId="21" priority="1338"/>
-    <cfRule type="duplicateValues" dxfId="20" priority="1339" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="1338"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1339" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:L1">
-    <cfRule type="duplicateValues" dxfId="19" priority="1336"/>
-    <cfRule type="duplicateValues" dxfId="18" priority="1337" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D463:D465">
-    <cfRule type="duplicateValues" dxfId="17" priority="1570"/>
-    <cfRule type="duplicateValues" dxfId="16" priority="1571"/>
-    <cfRule type="duplicateValues" dxfId="15" priority="1572"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="1573"/>
-    <cfRule type="duplicateValues" dxfId="13" priority="1574"/>
-    <cfRule type="duplicateValues" dxfId="12" priority="1575"/>
-    <cfRule type="duplicateValues" dxfId="11" priority="1576" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="1577" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A455:A462">
-    <cfRule type="duplicateValues" dxfId="9" priority="1587"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D450:D454">
-    <cfRule type="duplicateValues" dxfId="8" priority="1589"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="1590"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="1591"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="1592"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="1593"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="1594"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="1595" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="1596" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A448:A449">
-    <cfRule type="duplicateValues" dxfId="0" priority="1597"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="1336"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1337" stopIfTrue="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Data: refresh Nexlev + Viomi inventory inputs (Amazon, ledger, AMPM snapshot)
- inventory_amazon_nexlev.csv  (127 rows)
- inventory_amazon_viomi.csv   (200 rows)
- inventory_ledger_nexlev.csv  (748 rows)
- inventory_ledger_viomi.csv   (503 rows)
- inventory_snapshot_nexlev.xlsx (421 rows, B2B-AMPM channel intact)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/inventory_snapshot_nexlev.xlsx
+++ b/data/input/inventory_snapshot_nexlev.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\inventory\Week 23\Nexlev\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F373F78-5980-4B62-B49C-92684D93C635}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -9814,23 +9814,23 @@
   </sheetData>
   <autoFilter ref="A1:L422" xr:uid="{76CBFB1B-DC23-4380-8138-4D6BFF18CBC5}"/>
   <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="A147:A151">
+    <cfRule type="duplicateValues" dxfId="7" priority="2088"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="duplicateValues" dxfId="7" priority="1873"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="1873"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:H1">
-    <cfRule type="duplicateValues" dxfId="6" priority="2084"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="2085" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="2084"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="2085" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1">
-    <cfRule type="duplicateValues" dxfId="4" priority="1871"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="1872" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="1871"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1872" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:L1">
-    <cfRule type="duplicateValues" dxfId="2" priority="1869"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="1870" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A147:A151">
-    <cfRule type="duplicateValues" dxfId="0" priority="2088"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="1869"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1870" stopIfTrue="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Inventory snapshots: swap Pipeline <-> Open Order labels
Operator flagged that in prior snapshots the labels were backwards:
- 'Pipeline' actually meant Open PO to China (not yet shipped)
- 'Open Order' actually meant in-transit stock from China (Pipeline)

Refreshed inventory snapshots for all 4 accounts with corrected labels:
- Nexlev:      Pipeline    5 rows /  7,401 | Open Order  9 rows / 12,052
              (relabelled 9 rows with Channel='0' -> 'Open Order')
- Audio Array: Pipeline   11 rows /  6,390 | Open Order 34 rows / 26,295
- WM:          Pipeline    0 rows /      0 | Open Order  2 rows /  2,000
- Tonor:       Pipeline    0 rows /      0 | Open Order  1 row  /     80

CB Replenishment service reads Pipeline channel for 'china_in_transit'
metric, so this correction directly impacts CB PO Req calculations.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/inventory_snapshot_nexlev.xlsx
+++ b/data/input/inventory_snapshot_nexlev.xlsx
@@ -9148,7 +9148,7 @@
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K242" t="inlineStr"/>
@@ -9184,7 +9184,7 @@
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K243" t="inlineStr"/>
@@ -9220,7 +9220,7 @@
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K244" t="inlineStr"/>
@@ -9256,7 +9256,7 @@
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K245" t="inlineStr"/>
@@ -9292,7 +9292,7 @@
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K246" t="inlineStr"/>
@@ -9328,7 +9328,7 @@
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K247" t="inlineStr"/>
@@ -9364,7 +9364,7 @@
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K248" t="inlineStr"/>
@@ -9400,7 +9400,7 @@
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K249" t="inlineStr"/>
@@ -9436,7 +9436,7 @@
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K250" t="inlineStr"/>
@@ -9472,7 +9472,7 @@
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K251" t="inlineStr"/>
@@ -9508,7 +9508,7 @@
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K252" t="inlineStr"/>
@@ -9544,7 +9544,7 @@
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K253" t="inlineStr"/>
@@ -9580,7 +9580,7 @@
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K254" t="inlineStr"/>
@@ -9616,7 +9616,7 @@
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>Open Order</t>
         </is>
       </c>
       <c r="K255" t="inlineStr"/>

</xml_diff>